<commit_message>
WIP: modelo Micron (MU) apos primeira rodada do construtor
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019CsKrArZ7jEHMg4re9nbdn
</commit_message>
<xml_diff>
--- a/models/Micron_MU_modelo_out26.xlsx
+++ b/models/Micron_MU_modelo_out26.xlsx
@@ -33,7 +33,7 @@
 <file path=xl/comments10.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
-    <author>Unknown Author</author>
+    <author>LF</author>
   </authors>
   <commentList>
     <comment ref="D6" authorId="0">
@@ -93,6 +93,18 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">estimado/derivado: PR rounds to $1.05B</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D16" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">estimado/derivado: derived GAAP NI / GAAP EPS</t>
         </r>
       </text>
     </comment>
@@ -156,7 +168,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E36" authorId="0">
+    <comment ref="E16" authorId="0">
       <text>
         <r>
           <rPr>
@@ -164,7 +176,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">estimado</t>
+          <t xml:space="preserve">estimado/derivado: derived GAAP NI / GAAP EPS</t>
         </r>
       </text>
     </comment>
@@ -193,6 +205,18 @@
       </text>
     </comment>
     <comment ref="E39" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">estimado</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E40" authorId="0">
       <text>
         <r>
           <rPr>
@@ -252,7 +276,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F36" authorId="0">
+    <comment ref="F16" authorId="0">
       <text>
         <r>
           <rPr>
@@ -260,7 +284,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">estimado</t>
+          <t xml:space="preserve">estimado/derivado: derived non-GAAP NI / non-GAAP EPS</t>
         </r>
       </text>
     </comment>
@@ -289,6 +313,18 @@
       </text>
     </comment>
     <comment ref="F39" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">estimado</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F40" authorId="0">
       <text>
         <r>
           <rPr>
@@ -360,7 +396,19 @@
         </r>
       </text>
     </comment>
-    <comment ref="G19" authorId="0">
+    <comment ref="G16" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">estimado/derivado: derived GAAP NI / GAAP EPS</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G20" authorId="0">
       <text>
         <r>
           <rPr>
@@ -372,7 +420,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G20" authorId="0">
+    <comment ref="G21" authorId="0">
       <text>
         <r>
           <rPr>
@@ -432,7 +480,19 @@
         </r>
       </text>
     </comment>
-    <comment ref="H36" authorId="0">
+    <comment ref="H16" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">estimado/derivado: derived non-GAAP NI / non-GAAP EPS</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H37" authorId="0">
       <text>
         <r>
           <rPr>
@@ -444,7 +504,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H37" authorId="0">
+    <comment ref="H38" authorId="0">
       <text>
         <r>
           <rPr>
@@ -516,6 +576,18 @@
         </r>
       </text>
     </comment>
+    <comment ref="I16" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">estimado/derivado: derived non-GAAP NI / non-GAAP EPS</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="J6" authorId="0">
       <text>
         <r>
@@ -560,11 +632,23 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
+          <t xml:space="preserve">estimado/derivado: 3Q26 PR year-ago column shows 1,125; matches GAAP NI/EPS (1,890/1.68)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J17" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
           <t xml:space="preserve">estimado/derivado: remarks: $2.7B (rounded)</t>
         </r>
       </text>
     </comment>
-    <comment ref="J17" authorId="0">
+    <comment ref="J18" authorId="0">
       <text>
         <r>
           <rPr>
@@ -600,7 +684,19 @@
         </r>
       </text>
     </comment>
-    <comment ref="K19" authorId="0">
+    <comment ref="K16" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">estimado/derivado: derived non-GAAP NI / non-GAAP EPS</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K20" authorId="0">
       <text>
         <r>
           <rPr>
@@ -612,7 +708,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K34" authorId="0">
+    <comment ref="K35" authorId="0">
       <text>
         <r>
           <rPr>
@@ -668,7 +764,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">estimado/derivado: derived CFO 8,411 - adjusted FCF ~3,900</t>
+          <t xml:space="preserve">estimado/derivado: derived non-GAAP NI / non-GAAP EPS</t>
         </r>
       </text>
     </comment>
@@ -680,7 +776,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">estimado/derivado: remarks: $3.9B record (rounded)</t>
+          <t xml:space="preserve">estimado/derivado: derived CFO 8,411 - adjusted FCF ~3,900</t>
         </r>
       </text>
     </comment>
@@ -692,11 +788,11 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">estimado/derivado: derived debt 11.8B + 'net cash balance over $250M'</t>
+          <t xml:space="preserve">estimado/derivado: remarks: $3.9B record (rounded)</t>
         </r>
       </text>
     </comment>
-    <comment ref="L31" authorId="0">
+    <comment ref="L19" authorId="0">
       <text>
         <r>
           <rPr>
@@ -704,7 +800,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">estimado</t>
+          <t xml:space="preserve">estimado/derivado: derived debt 11.8B + 'net cash balance over $250M'</t>
         </r>
       </text>
     </comment>
@@ -733,6 +829,18 @@
       </text>
     </comment>
     <comment ref="L34" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">estimado</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L35" authorId="0">
       <text>
         <r>
           <rPr>
@@ -780,7 +888,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M16" authorId="0">
+    <comment ref="M17" authorId="0">
       <text>
         <r>
           <rPr>
@@ -792,7 +900,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M17" authorId="0">
+    <comment ref="M18" authorId="0">
       <text>
         <r>
           <rPr>
@@ -801,18 +909,6 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">estimado/derivado: PR: $6.9B (rounded)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M32" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">estimado</t>
         </r>
       </text>
     </comment>
@@ -829,6 +925,18 @@
       </text>
     </comment>
     <comment ref="M34" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">estimado</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M35" authorId="0">
       <text>
         <r>
           <rPr>
@@ -864,7 +972,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N16" authorId="0">
+    <comment ref="N17" authorId="0">
       <text>
         <r>
           <rPr>
@@ -876,7 +984,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N17" authorId="0">
+    <comment ref="N18" authorId="0">
       <text>
         <r>
           <rPr>
@@ -888,7 +996,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N19" authorId="0">
+    <comment ref="N20" authorId="0">
       <text>
         <r>
           <rPr>
@@ -960,7 +1068,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O16" authorId="0">
+    <comment ref="O17" authorId="0">
       <text>
         <r>
           <rPr>
@@ -972,7 +1080,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O17" authorId="0">
+    <comment ref="O18" authorId="0">
       <text>
         <r>
           <rPr>
@@ -984,7 +1092,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O19" authorId="0">
+    <comment ref="O20" authorId="0">
       <text>
         <r>
           <rPr>
@@ -1040,7 +1148,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">EPS x ~1.150 mn acoes (guia)</t>
+          <t xml:space="preserve">EPS x acoes guiadas (sanity)</t>
         </r>
       </text>
     </comment>
@@ -1064,11 +1172,23 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
+          <t xml:space="preserve">~1.150 mn acoes diluidas (call 4T26)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="P17" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
           <t xml:space="preserve">~11,5 bi; 1S27 ~25 bi; 2S maior</t>
         </r>
       </text>
     </comment>
-    <comment ref="P21" authorId="0">
+    <comment ref="P22" authorId="0">
       <text>
         <r>
           <rPr>
@@ -1087,7 +1207,7 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
-    <author>Unknown Author</author>
+    <author>LF</author>
   </authors>
   <commentList>
     <comment ref="B13" authorId="0">
@@ -1373,7 +1493,7 @@
 <file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
-    <author>Unknown Author</author>
+    <author>LF</author>
   </authors>
   <commentList>
     <comment ref="F6" authorId="0">
@@ -1491,7 +1611,7 @@
 <file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
-    <author>Unknown Author</author>
+    <author>LF</author>
   </authors>
   <commentList>
     <comment ref="D42" authorId="0">
@@ -1573,7 +1693,7 @@
 <file path=xl/comments5.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
-    <author>Unknown Author</author>
+    <author>LF</author>
   </authors>
   <commentList>
     <comment ref="D26" authorId="0">
@@ -1619,7 +1739,7 @@
 <file path=xl/comments6.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
-    <author>Unknown Author</author>
+    <author>LF</author>
   </authors>
   <commentList>
     <comment ref="D28" authorId="0">
@@ -1737,7 +1857,7 @@
 <file path=xl/comments7.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
-    <author>Unknown Author</author>
+    <author>LF</author>
   </authors>
   <commentList>
     <comment ref="H44" authorId="0">
@@ -1759,7 +1879,7 @@
 <file path=xl/comments9.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
-    <author>Unknown Author</author>
+    <author>LF</author>
   </authors>
   <commentList>
     <comment ref="D24" authorId="0">
@@ -2223,7 +2343,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1335" uniqueCount="994">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1336" uniqueCount="994">
   <si>
     <t xml:space="preserve">Micron Technology (MU US) - Resumo do modelo</t>
   </si>
@@ -6484,28 +6604,28 @@
       <c r="B30" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D30" s="20" t="n">
-        <f aca="false">Multiplos!$D$10/DRE!F16</f>
-        <v>122.475892602378</v>
+      <c r="D30" s="20" t="str">
+        <f aca="false">IF(Multiplos!$D$10/DRE!F16&gt;100,"n.m.",Multiplos!$D$10/DRE!F16)</f>
+        <v>n.m.</v>
       </c>
       <c r="E30" s="20" t="n">
-        <f aca="false">Multiplos!$D$10/DRE!G16</f>
+        <f aca="false">IF(Multiplos!$D$10/DRE!G16&gt;100,"n.m.",Multiplos!$D$10/DRE!G16)</f>
         <v>61.3933897141596</v>
       </c>
       <c r="F30" s="20" t="n">
-        <f aca="false">Multiplos!$D$10/DRE!H16</f>
+        <f aca="false">IF(Multiplos!$D$10/DRE!H16&gt;100,"n.m.",Multiplos!$D$10/DRE!H16)</f>
         <v>10.2217966097958</v>
       </c>
       <c r="G30" s="20" t="n">
-        <f aca="false">Multiplos!$D$10/DRE!I16</f>
+        <f aca="false">IF(Multiplos!$D$10/DRE!I16&gt;100,"n.m.",Multiplos!$D$10/DRE!I16)</f>
         <v>4.64676872371512</v>
       </c>
       <c r="H30" s="20" t="n">
-        <f aca="false">Multiplos!$D$10/DRE!J16</f>
+        <f aca="false">IF(Multiplos!$D$10/DRE!J16&gt;100,"n.m.",Multiplos!$D$10/DRE!J16)</f>
         <v>4.20087012475494</v>
       </c>
       <c r="I30" s="20" t="n">
-        <f aca="false">Multiplos!$D$10/DRE!K16</f>
+        <f aca="false">IF(Multiplos!$D$10/DRE!K16&gt;100,"n.m.",Multiplos!$D$10/DRE!K16)</f>
         <v>6.32274649676289</v>
       </c>
     </row>
@@ -6513,28 +6633,28 @@
       <c r="B31" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D31" s="20" t="n">
-        <f aca="false">Premissas!$I$203/DRE!F39</f>
-        <v>804.276923076923</v>
-      </c>
-      <c r="E31" s="20" t="n">
-        <f aca="false">Premissas!$I$203/DRE!G39</f>
-        <v>126.123039806996</v>
+      <c r="D31" s="20" t="str">
+        <f aca="false">IF(Premissas!$I$203/DRE!F39&gt;100,"n.m.",Premissas!$I$203/DRE!F39)</f>
+        <v>n.m.</v>
+      </c>
+      <c r="E31" s="20" t="str">
+        <f aca="false">IF(Premissas!$I$203/DRE!G39&gt;100,"n.m.",Premissas!$I$203/DRE!G39)</f>
+        <v>n.m.</v>
       </c>
       <c r="F31" s="20" t="n">
-        <f aca="false">Premissas!$I$203/DRE!H39</f>
+        <f aca="false">IF(Premissas!$I$203/DRE!H39&gt;100,"n.m.",Premissas!$I$203/DRE!H39)</f>
         <v>13.8448093220339</v>
       </c>
       <c r="G31" s="20" t="n">
-        <f aca="false">Premissas!$I$203/DRE!I39</f>
+        <f aca="false">IF(Premissas!$I$203/DRE!I39&gt;100,"n.m.",Premissas!$I$203/DRE!I39)</f>
         <v>5.94896038635783</v>
       </c>
       <c r="H31" s="20" t="n">
-        <f aca="false">Premissas!$I$203/DRE!J39</f>
+        <f aca="false">IF(Premissas!$I$203/DRE!J39&gt;100,"n.m.",Premissas!$I$203/DRE!J39)</f>
         <v>4.93088770339068</v>
       </c>
       <c r="I31" s="20" t="n">
-        <f aca="false">Premissas!$I$203/DRE!K39</f>
+        <f aca="false">IF(Premissas!$I$203/DRE!K39&gt;100,"n.m.",Premissas!$I$203/DRE!K39)</f>
         <v>6.79913267574938</v>
       </c>
     </row>
@@ -6770,7 +6890,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:P53"/>
+  <dimension ref="B1:P54"/>
   <sheetFormatPr defaultColWidth="8.75390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -7240,7 +7360,7 @@
         <v>38400</v>
       </c>
       <c r="P13" s="47" t="n">
-        <f aca="false">P14*1150</f>
+        <f aca="false">P14*P16</f>
         <v>43872.5</v>
       </c>
     </row>
@@ -7333,132 +7453,132 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="4" t="s">
-        <v>488</v>
+      <c r="B16" s="2" t="s">
+        <v>392</v>
       </c>
       <c r="D16" s="32" t="n">
-        <v>1730</v>
+        <v>1098</v>
       </c>
       <c r="E16" s="32" t="n">
-        <v>1250</v>
+        <v>1117</v>
       </c>
       <c r="F16" s="32" t="n">
-        <v>2057</v>
+        <v>1132</v>
       </c>
       <c r="G16" s="32" t="n">
-        <v>3080</v>
+        <v>1123</v>
       </c>
       <c r="H16" s="32" t="n">
-        <v>3130</v>
+        <v>1140</v>
       </c>
       <c r="I16" s="32" t="n">
-        <v>3090</v>
+        <v>1141</v>
       </c>
       <c r="J16" s="32" t="n">
-        <v>2700</v>
+        <v>1125</v>
       </c>
       <c r="K16" s="32" t="n">
-        <v>4930</v>
+        <v>1145</v>
       </c>
       <c r="L16" s="32" t="n">
-        <v>4500</v>
+        <v>1146</v>
       </c>
       <c r="M16" s="32" t="n">
-        <v>5000</v>
+        <v>1142</v>
       </c>
       <c r="N16" s="32" t="n">
-        <v>7100</v>
+        <v>1145</v>
       </c>
       <c r="O16" s="32" t="n">
-        <v>10770</v>
+        <v>1147</v>
       </c>
       <c r="P16" s="32" t="n">
-        <v>11500</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="4" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="D17" s="32" t="n">
-        <v>-333</v>
+        <v>1730</v>
       </c>
       <c r="E17" s="32" t="n">
-        <v>-29</v>
+        <v>1250</v>
       </c>
       <c r="F17" s="32" t="n">
-        <v>425</v>
+        <v>2057</v>
       </c>
       <c r="G17" s="32" t="n">
-        <v>323</v>
+        <v>3080</v>
       </c>
       <c r="H17" s="32" t="n">
-        <v>112</v>
+        <v>3130</v>
       </c>
       <c r="I17" s="32" t="n">
-        <v>857</v>
+        <v>3090</v>
       </c>
       <c r="J17" s="32" t="n">
-        <v>1900</v>
+        <v>2700</v>
       </c>
       <c r="K17" s="32" t="n">
-        <v>803</v>
+        <v>4930</v>
       </c>
       <c r="L17" s="32" t="n">
-        <v>3900</v>
+        <v>4500</v>
       </c>
       <c r="M17" s="32" t="n">
-        <v>6900</v>
+        <v>5000</v>
       </c>
       <c r="N17" s="32" t="n">
-        <v>18300</v>
+        <v>7100</v>
       </c>
       <c r="O17" s="32" t="n">
-        <v>33200</v>
-      </c>
-      <c r="P17" s="50" t="s">
-        <v>173</v>
+        <v>10770</v>
+      </c>
+      <c r="P17" s="32" t="n">
+        <v>11500</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="4" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="D18" s="32" t="n">
-        <v>9840</v>
+        <v>-333</v>
       </c>
       <c r="E18" s="32" t="n">
-        <v>9720</v>
+        <v>-29</v>
       </c>
       <c r="F18" s="32" t="n">
-        <v>9220</v>
+        <v>425</v>
       </c>
       <c r="G18" s="32" t="n">
-        <v>9160</v>
+        <v>323</v>
       </c>
       <c r="H18" s="32" t="n">
-        <v>8750</v>
+        <v>112</v>
       </c>
       <c r="I18" s="32" t="n">
-        <v>9600</v>
+        <v>857</v>
       </c>
       <c r="J18" s="32" t="n">
-        <v>12200</v>
+        <v>1900</v>
       </c>
       <c r="K18" s="32" t="n">
-        <v>11940</v>
+        <v>803</v>
       </c>
       <c r="L18" s="32" t="n">
-        <v>12050</v>
+        <v>3900</v>
       </c>
       <c r="M18" s="32" t="n">
-        <v>16700</v>
+        <v>6900</v>
       </c>
       <c r="N18" s="32" t="n">
-        <v>30200</v>
+        <v>18300</v>
       </c>
       <c r="O18" s="32" t="n">
-        <v>73480</v>
+        <v>33200</v>
       </c>
       <c r="P18" s="50" t="s">
         <v>173</v>
@@ -7466,43 +7586,43 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="4" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="D19" s="32" t="n">
-        <v>13505</v>
+        <v>9840</v>
       </c>
       <c r="E19" s="32" t="n">
-        <v>13722</v>
+        <v>9720</v>
       </c>
       <c r="F19" s="32" t="n">
-        <v>13258</v>
+        <v>9220</v>
       </c>
       <c r="G19" s="32" t="n">
-        <v>13400</v>
+        <v>9160</v>
       </c>
       <c r="H19" s="32" t="n">
-        <v>13800</v>
-      </c>
-      <c r="I19" s="50" t="s">
-        <v>173</v>
+        <v>8750</v>
+      </c>
+      <c r="I19" s="32" t="n">
+        <v>9600</v>
       </c>
       <c r="J19" s="32" t="n">
-        <v>15500</v>
+        <v>12200</v>
       </c>
       <c r="K19" s="32" t="n">
-        <v>14600</v>
+        <v>11940</v>
       </c>
       <c r="L19" s="32" t="n">
-        <v>11800</v>
+        <v>12050</v>
       </c>
       <c r="M19" s="32" t="n">
-        <v>10100</v>
+        <v>16700</v>
       </c>
       <c r="N19" s="32" t="n">
-        <v>5700</v>
+        <v>30200</v>
       </c>
       <c r="O19" s="32" t="n">
-        <v>5179</v>
+        <v>73480</v>
       </c>
       <c r="P19" s="50" t="s">
         <v>173</v>
@@ -7510,43 +7630,43 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="4" t="s">
-        <v>492</v>
-      </c>
-      <c r="D20" s="50" t="s">
+        <v>491</v>
+      </c>
+      <c r="D20" s="32" t="n">
+        <v>13505</v>
+      </c>
+      <c r="E20" s="32" t="n">
+        <v>13722</v>
+      </c>
+      <c r="F20" s="32" t="n">
+        <v>13258</v>
+      </c>
+      <c r="G20" s="32" t="n">
+        <v>13400</v>
+      </c>
+      <c r="H20" s="32" t="n">
+        <v>13800</v>
+      </c>
+      <c r="I20" s="50" t="s">
         <v>173</v>
       </c>
-      <c r="E20" s="50" t="s">
-        <v>173</v>
-      </c>
-      <c r="F20" s="50" t="s">
-        <v>173</v>
-      </c>
-      <c r="G20" s="34" t="n">
-        <v>158</v>
-      </c>
-      <c r="H20" s="34" t="n">
-        <v>149</v>
-      </c>
-      <c r="I20" s="34" t="n">
-        <v>158</v>
-      </c>
-      <c r="J20" s="50" t="s">
-        <v>173</v>
-      </c>
-      <c r="K20" s="34" t="n">
-        <v>124</v>
-      </c>
-      <c r="L20" s="34" t="n">
-        <v>126</v>
-      </c>
-      <c r="M20" s="34" t="n">
-        <v>123</v>
-      </c>
-      <c r="N20" s="34" t="n">
-        <v>120</v>
-      </c>
-      <c r="O20" s="34" t="n">
-        <v>129</v>
+      <c r="J20" s="32" t="n">
+        <v>15500</v>
+      </c>
+      <c r="K20" s="32" t="n">
+        <v>14600</v>
+      </c>
+      <c r="L20" s="32" t="n">
+        <v>11800</v>
+      </c>
+      <c r="M20" s="32" t="n">
+        <v>10100</v>
+      </c>
+      <c r="N20" s="32" t="n">
+        <v>5700</v>
+      </c>
+      <c r="O20" s="32" t="n">
+        <v>5179</v>
       </c>
       <c r="P20" s="50" t="s">
         <v>173</v>
@@ -7554,557 +7674,601 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="4" t="s">
+        <v>492</v>
+      </c>
+      <c r="D21" s="50" t="s">
+        <v>173</v>
+      </c>
+      <c r="E21" s="50" t="s">
+        <v>173</v>
+      </c>
+      <c r="F21" s="50" t="s">
+        <v>173</v>
+      </c>
+      <c r="G21" s="34" t="n">
+        <v>158</v>
+      </c>
+      <c r="H21" s="34" t="n">
+        <v>149</v>
+      </c>
+      <c r="I21" s="34" t="n">
+        <v>158</v>
+      </c>
+      <c r="J21" s="50" t="s">
+        <v>173</v>
+      </c>
+      <c r="K21" s="34" t="n">
+        <v>124</v>
+      </c>
+      <c r="L21" s="34" t="n">
+        <v>126</v>
+      </c>
+      <c r="M21" s="34" t="n">
+        <v>123</v>
+      </c>
+      <c r="N21" s="34" t="n">
+        <v>120</v>
+      </c>
+      <c r="O21" s="34" t="n">
+        <v>129</v>
+      </c>
+      <c r="P21" s="50" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="4" t="s">
         <v>222</v>
       </c>
-      <c r="D21" s="46" t="n">
+      <c r="D22" s="46" t="n">
         <v>0.115</v>
       </c>
-      <c r="E21" s="46" t="n">
+      <c r="E22" s="46" t="n">
         <v>0.115</v>
       </c>
-      <c r="F21" s="46" t="n">
+      <c r="F22" s="46" t="n">
         <v>0.115</v>
       </c>
-      <c r="G21" s="46" t="n">
+      <c r="G22" s="46" t="n">
         <v>0.115</v>
       </c>
-      <c r="H21" s="46" t="n">
+      <c r="H22" s="46" t="n">
         <v>0.115</v>
       </c>
-      <c r="I21" s="46" t="n">
+      <c r="I22" s="46" t="n">
         <v>0.115</v>
       </c>
-      <c r="J21" s="46" t="n">
+      <c r="J22" s="46" t="n">
         <v>0.115</v>
       </c>
-      <c r="K21" s="46" t="n">
+      <c r="K22" s="46" t="n">
         <v>0.115</v>
       </c>
-      <c r="L21" s="46" t="n">
+      <c r="L22" s="46" t="n">
         <v>0.115</v>
       </c>
-      <c r="M21" s="46" t="n">
+      <c r="M22" s="46" t="n">
         <v>0.115</v>
       </c>
-      <c r="N21" s="46" t="n">
+      <c r="N22" s="46" t="n">
         <v>0.15</v>
       </c>
-      <c r="O21" s="46" t="n">
+      <c r="O22" s="46" t="n">
         <v>0.15</v>
       </c>
-      <c r="P21" s="46" t="n">
+      <c r="P22" s="46" t="n">
         <v>0.15</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="3" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="3" t="s">
         <v>493</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="4" t="s">
-        <v>494</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>495</v>
-      </c>
-      <c r="D24" s="51" t="s">
-        <v>496</v>
-      </c>
-      <c r="E24" s="51" t="s">
-        <v>497</v>
-      </c>
-      <c r="F24" s="51" t="s">
-        <v>498</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="H24" s="51" t="s">
-        <v>499</v>
-      </c>
-      <c r="I24" s="51" t="s">
-        <v>500</v>
-      </c>
-      <c r="J24" s="51" t="s">
-        <v>501</v>
-      </c>
-      <c r="K24" s="51" t="s">
-        <v>502</v>
-      </c>
-      <c r="L24" s="51" t="s">
-        <v>503</v>
-      </c>
-      <c r="M24" s="51" t="s">
-        <v>504</v>
-      </c>
-      <c r="N24" s="51" t="s">
-        <v>505</v>
-      </c>
-      <c r="O24" s="51" t="s">
-        <v>506</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="4" t="s">
-        <v>507</v>
+        <v>494</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>495</v>
       </c>
       <c r="D25" s="51" t="s">
-        <v>508</v>
+        <v>496</v>
       </c>
       <c r="E25" s="51" t="s">
-        <v>509</v>
+        <v>497</v>
       </c>
       <c r="F25" s="51" t="s">
-        <v>510</v>
+        <v>498</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>173</v>
       </c>
       <c r="H25" s="51" t="s">
-        <v>511</v>
+        <v>499</v>
       </c>
       <c r="I25" s="51" t="s">
-        <v>512</v>
+        <v>500</v>
       </c>
       <c r="J25" s="51" t="s">
-        <v>513</v>
+        <v>501</v>
       </c>
       <c r="K25" s="51" t="s">
-        <v>514</v>
+        <v>502</v>
       </c>
       <c r="L25" s="51" t="s">
-        <v>515</v>
+        <v>503</v>
       </c>
       <c r="M25" s="51" t="s">
-        <v>516</v>
+        <v>504</v>
       </c>
       <c r="N25" s="51" t="s">
-        <v>517</v>
+        <v>505</v>
       </c>
       <c r="O25" s="51" t="s">
-        <v>518</v>
+        <v>506</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="4" t="s">
-        <v>519</v>
+        <v>507</v>
       </c>
       <c r="D26" s="51" t="s">
-        <v>520</v>
+        <v>508</v>
       </c>
       <c r="E26" s="51" t="s">
-        <v>521</v>
+        <v>509</v>
       </c>
       <c r="F26" s="51" t="s">
-        <v>522</v>
+        <v>510</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>173</v>
       </c>
       <c r="H26" s="51" t="s">
-        <v>523</v>
+        <v>511</v>
       </c>
       <c r="I26" s="51" t="s">
-        <v>524</v>
+        <v>512</v>
       </c>
       <c r="J26" s="51" t="s">
-        <v>525</v>
+        <v>513</v>
       </c>
       <c r="K26" s="51" t="s">
-        <v>526</v>
+        <v>514</v>
       </c>
       <c r="L26" s="51" t="s">
-        <v>527</v>
+        <v>515</v>
       </c>
       <c r="M26" s="51" t="s">
-        <v>528</v>
+        <v>516</v>
       </c>
       <c r="N26" s="51" t="s">
-        <v>504</v>
+        <v>517</v>
       </c>
       <c r="O26" s="51" t="s">
-        <v>529</v>
+        <v>518</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="4" t="s">
-        <v>530</v>
+        <v>519</v>
       </c>
       <c r="D27" s="51" t="s">
-        <v>531</v>
+        <v>520</v>
       </c>
       <c r="E27" s="51" t="s">
-        <v>532</v>
+        <v>521</v>
       </c>
       <c r="F27" s="51" t="s">
-        <v>531</v>
+        <v>522</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>173</v>
       </c>
       <c r="H27" s="51" t="s">
-        <v>533</v>
+        <v>523</v>
       </c>
       <c r="I27" s="51" t="s">
-        <v>534</v>
+        <v>524</v>
       </c>
       <c r="J27" s="51" t="s">
-        <v>535</v>
+        <v>525</v>
       </c>
       <c r="K27" s="51" t="s">
-        <v>536</v>
+        <v>526</v>
       </c>
       <c r="L27" s="51" t="s">
-        <v>537</v>
+        <v>527</v>
       </c>
       <c r="M27" s="51" t="s">
-        <v>538</v>
+        <v>528</v>
       </c>
       <c r="N27" s="51" t="s">
-        <v>539</v>
+        <v>504</v>
       </c>
       <c r="O27" s="51" t="s">
-        <v>540</v>
+        <v>529</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="4" t="s">
+        <v>530</v>
+      </c>
+      <c r="D28" s="51" t="s">
+        <v>531</v>
+      </c>
+      <c r="E28" s="51" t="s">
+        <v>532</v>
+      </c>
+      <c r="F28" s="51" t="s">
+        <v>531</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="H28" s="51" t="s">
+        <v>533</v>
+      </c>
+      <c r="I28" s="51" t="s">
+        <v>534</v>
+      </c>
+      <c r="J28" s="51" t="s">
+        <v>535</v>
+      </c>
+      <c r="K28" s="51" t="s">
+        <v>536</v>
+      </c>
+      <c r="L28" s="51" t="s">
+        <v>537</v>
+      </c>
+      <c r="M28" s="51" t="s">
+        <v>538</v>
+      </c>
+      <c r="N28" s="51" t="s">
+        <v>539</v>
+      </c>
+      <c r="O28" s="51" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="4" t="s">
         <v>541</v>
       </c>
-      <c r="D28" s="51" t="s">
+      <c r="D29" s="51" t="s">
         <v>542</v>
       </c>
-      <c r="E28" s="51" t="s">
+      <c r="E29" s="51" t="s">
         <v>543</v>
       </c>
-      <c r="F28" s="51" t="s">
+      <c r="F29" s="51" t="s">
         <v>544</v>
       </c>
-      <c r="G28" s="51" t="s">
+      <c r="G29" s="51" t="s">
         <v>545</v>
       </c>
-      <c r="H28" s="51" t="s">
+      <c r="H29" s="51" t="s">
         <v>546</v>
       </c>
-      <c r="I28" s="51" t="s">
+      <c r="I29" s="51" t="s">
         <v>547</v>
       </c>
-      <c r="J28" s="51" t="s">
+      <c r="J29" s="51" t="s">
         <v>548</v>
       </c>
-      <c r="K28" s="51" t="s">
+      <c r="K29" s="51" t="s">
         <v>549</v>
       </c>
-      <c r="L28" s="51" t="s">
+      <c r="L29" s="51" t="s">
         <v>550</v>
       </c>
-      <c r="M28" s="51" t="s">
+      <c r="M29" s="51" t="s">
         <v>551</v>
       </c>
-      <c r="N28" s="51" t="s">
+      <c r="N29" s="51" t="s">
         <v>552</v>
       </c>
-      <c r="O28" s="51" t="s">
+      <c r="O29" s="51" t="s">
         <v>553</v>
       </c>
-      <c r="P28" s="51" t="s">
+      <c r="P29" s="51" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="3" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="3" t="s">
         <v>555</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="4" t="s">
-        <v>556</v>
-      </c>
-      <c r="K31" s="32" t="n">
-        <v>4543</v>
-      </c>
-      <c r="L31" s="32" t="n">
-        <v>5300</v>
-      </c>
-      <c r="M31" s="32" t="n">
-        <v>7749</v>
-      </c>
-      <c r="N31" s="32" t="n">
-        <v>13769</v>
-      </c>
-      <c r="O31" s="32" t="n">
-        <v>16283</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="4" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="K32" s="32" t="n">
-        <v>1577</v>
+        <v>4543</v>
       </c>
       <c r="L32" s="32" t="n">
-        <v>2379</v>
+        <v>5300</v>
       </c>
       <c r="M32" s="32" t="n">
-        <v>5690</v>
+        <v>7749</v>
       </c>
       <c r="N32" s="32" t="n">
-        <v>11524</v>
+        <v>13769</v>
       </c>
       <c r="O32" s="32" t="n">
-        <v>18002</v>
+        <v>16283</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="4" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="K33" s="32" t="n">
-        <v>3760</v>
+        <v>1577</v>
       </c>
       <c r="L33" s="32" t="n">
-        <v>4300</v>
+        <v>2379</v>
       </c>
       <c r="M33" s="32" t="n">
-        <v>7700</v>
+        <v>5690</v>
       </c>
       <c r="N33" s="32" t="n">
-        <v>11521</v>
+        <v>11524</v>
       </c>
       <c r="O33" s="32" t="n">
-        <v>13114</v>
+        <v>18002</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="4" t="s">
+        <v>558</v>
+      </c>
+      <c r="K34" s="32" t="n">
+        <v>3760</v>
+      </c>
+      <c r="L34" s="32" t="n">
+        <v>4300</v>
+      </c>
+      <c r="M34" s="32" t="n">
+        <v>7700</v>
+      </c>
+      <c r="N34" s="32" t="n">
+        <v>11521</v>
+      </c>
+      <c r="O34" s="32" t="n">
+        <v>13114</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B35" s="4" t="s">
         <v>559</v>
       </c>
-      <c r="K34" s="32" t="n">
+      <c r="K35" s="32" t="n">
         <v>1435</v>
       </c>
-      <c r="L34" s="32" t="n">
+      <c r="L35" s="32" t="n">
         <v>1700</v>
       </c>
-      <c r="M34" s="32" t="n">
+      <c r="M35" s="32" t="n">
         <v>2700</v>
       </c>
-      <c r="N34" s="32" t="n">
+      <c r="N35" s="32" t="n">
         <v>4634</v>
       </c>
-      <c r="O34" s="32" t="n">
+      <c r="O35" s="32" t="n">
         <v>6824</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="3" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B36" s="3" t="s">
         <v>560</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="4" t="s">
-        <v>561</v>
-      </c>
-      <c r="D36" s="32" t="n">
-        <v>1737</v>
-      </c>
-      <c r="E36" s="32" t="n">
-        <v>2185</v>
-      </c>
-      <c r="F36" s="32" t="n">
-        <v>2570</v>
-      </c>
-      <c r="H36" s="32" t="n">
-        <v>4395</v>
-      </c>
-      <c r="I36" s="32" t="n">
-        <v>4564</v>
-      </c>
-      <c r="J36" s="32" t="n">
-        <v>5069</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="4" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="D37" s="32" t="n">
-        <v>1293</v>
+        <v>1737</v>
       </c>
       <c r="E37" s="32" t="n">
-        <v>1598</v>
+        <v>2185</v>
       </c>
       <c r="F37" s="32" t="n">
-        <v>1590</v>
+        <v>2570</v>
       </c>
       <c r="H37" s="32" t="n">
-        <v>1527</v>
+        <v>4395</v>
       </c>
       <c r="I37" s="32" t="n">
-        <v>1068</v>
+        <v>4564</v>
       </c>
       <c r="J37" s="32" t="n">
-        <v>1551</v>
+        <v>5069</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="4" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="D38" s="32" t="n">
-        <v>1037</v>
+        <v>1293</v>
       </c>
       <c r="E38" s="32" t="n">
-        <v>1111</v>
+        <v>1598</v>
       </c>
       <c r="F38" s="32" t="n">
-        <v>1290</v>
+        <v>1590</v>
+      </c>
+      <c r="H38" s="32" t="n">
+        <v>1527</v>
       </c>
       <c r="I38" s="32" t="n">
-        <v>1025</v>
+        <v>1068</v>
       </c>
       <c r="J38" s="32" t="n">
-        <v>1227</v>
+        <v>1551</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="4" t="s">
+        <v>563</v>
+      </c>
+      <c r="D39" s="32" t="n">
+        <v>1037</v>
+      </c>
+      <c r="E39" s="32" t="n">
+        <v>1111</v>
+      </c>
+      <c r="F39" s="32" t="n">
+        <v>1290</v>
+      </c>
+      <c r="I39" s="32" t="n">
+        <v>1025</v>
+      </c>
+      <c r="J39" s="32" t="n">
+        <v>1227</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B40" s="4" t="s">
         <v>564</v>
       </c>
-      <c r="D39" s="32" t="n">
+      <c r="D40" s="32" t="n">
         <v>653</v>
       </c>
-      <c r="E39" s="32" t="n">
+      <c r="E40" s="32" t="n">
         <v>905</v>
       </c>
-      <c r="F39" s="32" t="n">
+      <c r="F40" s="32" t="n">
         <v>1350</v>
       </c>
-      <c r="I39" s="32" t="n">
+      <c r="I40" s="32" t="n">
         <v>1392</v>
       </c>
-      <c r="J39" s="32" t="n">
+      <c r="J40" s="32" t="n">
         <v>1451</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="3" t="s">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B42" s="3" t="s">
         <v>565</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="4" t="s">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B43" s="4" t="s">
         <v>566</v>
       </c>
-      <c r="D42" s="47" t="n">
+      <c r="D43" s="47" t="n">
         <f aca="false">4*P5</f>
         <v>246000</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="4" t="s">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B44" s="4" t="s">
         <v>567</v>
       </c>
-      <c r="D43" s="18" t="n">
+      <c r="D44" s="18" t="n">
         <f aca="false">DRE!$I$5</f>
         <v>272846.642</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="2" t="s">
-        <v>568</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>569</v>
-      </c>
-      <c r="D44" s="16" t="n">
-        <f aca="false">D43/D42-1</f>
-        <v>0.109132691056911</v>
-      </c>
-    </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>569</v>
+      </c>
+      <c r="D45" s="16" t="n">
+        <f aca="false">D44/D43-1</f>
+        <v>0.109132691056911</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B46" s="2" t="s">
         <v>570</v>
       </c>
-      <c r="D45" s="48" t="n">
-        <f aca="false">D43/4</f>
+      <c r="D46" s="48" t="n">
+        <f aca="false">D44/4</f>
         <v>68211.6605</v>
       </c>
-      <c r="E45" s="16" t="n">
-        <f aca="false">D45/P5-1</f>
+      <c r="E46" s="16" t="n">
+        <f aca="false">D46/P5-1</f>
         <v>0.109132691056911</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B46" s="4" t="s">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B47" s="4" t="s">
         <v>571</v>
       </c>
-      <c r="D46" s="21" t="n">
+      <c r="D47" s="21" t="n">
         <f aca="false">P9</f>
         <v>0.8595</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="4" t="s">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B48" s="4" t="s">
         <v>572</v>
       </c>
-      <c r="D47" s="64" t="n">
+      <c r="D48" s="64" t="n">
         <f aca="false">DRE!$I$9</f>
         <v>0.868065076600796</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B48" s="4" t="s">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B49" s="4" t="s">
         <v>573</v>
       </c>
-      <c r="D48" s="53" t="n">
+      <c r="D49" s="53" t="n">
         <f aca="false">4*P14</f>
         <v>152.6</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B49" s="4" t="s">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B50" s="4" t="s">
         <v>574</v>
       </c>
-      <c r="D49" s="61" t="n">
+      <c r="D50" s="61" t="n">
         <f aca="false">DRE!$I$39</f>
         <v>175.755078550814</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B50" s="4" t="s">
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B51" s="4" t="s">
         <v>575</v>
       </c>
-      <c r="D50" s="18" t="n">
+      <c r="D51" s="18" t="n">
         <f aca="false">Premissas!$I$207</f>
         <v>275010</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="2" t="s">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B52" s="2" t="s">
         <v>576</v>
       </c>
-      <c r="D51" s="16" t="n">
-        <f aca="false">D43/D50-1</f>
+      <c r="D52" s="16" t="n">
+        <f aca="false">D44/D51-1</f>
         <v>-0.00786647031017052</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B52" s="4" t="s">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B53" s="4" t="s">
         <v>577</v>
       </c>
-      <c r="D52" s="61" t="n">
+      <c r="D53" s="61" t="n">
         <f aca="false">Premissas!$I$208</f>
         <v>176.15</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B53" s="2" t="s">
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B54" s="2" t="s">
         <v>576</v>
       </c>
-      <c r="D53" s="16" t="n">
-        <f aca="false">D49/D52-1</f>
+      <c r="D54" s="16" t="n">
+        <f aca="false">D50/D53-1</f>
         <v>-0.00224196110806751</v>
       </c>
     </row>
@@ -15963,40 +16127,40 @@
       <c r="B28" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="E28" s="16" t="n">
-        <f aca="false">IF(D26&lt;=0,"n.m.",E26/D26-1)</f>
-        <v>-1.67146310579026</v>
+      <c r="E28" s="16" t="str">
+        <f aca="false">IF(OR(D26&lt;=0,E26&lt;=0),"n.m.",E26/D26-1)</f>
+        <v>n.m.</v>
       </c>
       <c r="F28" s="16" t="str">
-        <f aca="false">IF(E26&lt;=0,"n.m.",F26/E26-1)</f>
+        <f aca="false">IF(OR(E26&lt;=0,F26&lt;=0),"n.m.",F26/E26-1)</f>
         <v>n.m.</v>
       </c>
       <c r="G28" s="16" t="n">
-        <f aca="false">IF(F26&lt;=0,"n.m.",G26/F26-1)</f>
+        <f aca="false">IF(OR(F26&lt;=0,G26&lt;=0),"n.m.",G26/F26-1)</f>
         <v>9.97557840616967</v>
       </c>
       <c r="H28" s="16" t="n">
-        <f aca="false">IF(G26&lt;=0,"n.m.",H26/G26-1)</f>
+        <f aca="false">IF(OR(G26&lt;=0,H26&lt;=0),"n.m.",H26/G26-1)</f>
         <v>8.95069680290432</v>
       </c>
       <c r="I28" s="16" t="n">
-        <f aca="false">IF(H26&lt;=0,"n.m.",I26/H26-1)</f>
+        <f aca="false">IF(OR(H26&lt;=0,I26&lt;=0),"n.m.",I26/H26-1)</f>
         <v>1.2862442946411</v>
       </c>
       <c r="J28" s="16" t="n">
-        <f aca="false">IF(I26&lt;=0,"n.m.",J26/I26-1)</f>
+        <f aca="false">IF(OR(I26&lt;=0,J26&lt;=0),"n.m.",J26/I26-1)</f>
         <v>0.0965556888123154</v>
       </c>
       <c r="K28" s="16" t="n">
-        <f aca="false">IF(J26&lt;=0,"n.m.",K26/J26-1)</f>
+        <f aca="false">IF(OR(J26&lt;=0,K26&lt;=0),"n.m.",K26/J26-1)</f>
         <v>-0.368953733213617</v>
       </c>
       <c r="L28" s="16" t="n">
-        <f aca="false">IF(K26&lt;=0,"n.m.",L26/K26-1)</f>
+        <f aca="false">IF(OR(K26&lt;=0,L26&lt;=0),"n.m.",L26/K26-1)</f>
         <v>-0.328914326376645</v>
       </c>
       <c r="M28" s="16" t="n">
-        <f aca="false">IF(L26&lt;=0,"n.m.",M26/L26-1)</f>
+        <f aca="false">IF(OR(L26&lt;=0,M26&lt;=0),"n.m.",M26/L26-1)</f>
         <v>0.354035908022662</v>
       </c>
     </row>
@@ -16087,40 +16251,40 @@
       <c r="B32" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="E32" s="16" t="n">
-        <f aca="false">IF(D31&lt;=0,"n.m.",E31/D31-1)</f>
-        <v>-1.68903225806452</v>
+      <c r="E32" s="16" t="str">
+        <f aca="false">IF(OR(D31&lt;=0,E31&lt;=0),"n.m.",E31/D31-1)</f>
+        <v>n.m.</v>
       </c>
       <c r="F32" s="16" t="str">
-        <f aca="false">IF(E31&lt;=0,"n.m.",F31/E31-1)</f>
+        <f aca="false">IF(OR(E31&lt;=0,F31&lt;=0),"n.m.",F31/E31-1)</f>
         <v>n.m.</v>
       </c>
       <c r="G32" s="16" t="n">
-        <f aca="false">IF(F31&lt;=0,"n.m.",G31/F31-1)</f>
+        <f aca="false">IF(OR(F31&lt;=0,G31&lt;=0),"n.m.",G31/F31-1)</f>
         <v>9.84285714285714</v>
       </c>
       <c r="H32" s="16" t="n">
-        <f aca="false">IF(G31&lt;=0,"n.m.",H31/G31-1)</f>
+        <f aca="false">IF(OR(G31&lt;=0,H31&lt;=0),"n.m.",H31/G31-1)</f>
         <v>8.7931488801054</v>
       </c>
       <c r="I32" s="16" t="n">
-        <f aca="false">IF(H31&lt;=0,"n.m.",I31/H31-1)</f>
+        <f aca="false">IF(OR(H31&lt;=0,I31&lt;=0),"n.m.",I31/H31-1)</f>
         <v>1.34421401846379</v>
       </c>
       <c r="J32" s="16" t="n">
-        <f aca="false">IF(I31&lt;=0,"n.m.",J31/I31-1)</f>
+        <f aca="false">IF(OR(I31&lt;=0,J31&lt;=0),"n.m.",J31/I31-1)</f>
         <v>0.206033170788208</v>
       </c>
       <c r="K32" s="16" t="n">
-        <f aca="false">IF(J31&lt;=0,"n.m.",K31/J31-1)</f>
+        <f aca="false">IF(OR(J31&lt;=0,K31&lt;=0),"n.m.",K31/J31-1)</f>
         <v>-0.279604008027992</v>
       </c>
       <c r="L32" s="16" t="n">
-        <f aca="false">IF(K31&lt;=0,"n.m.",L31/K31-1)</f>
+        <f aca="false">IF(OR(K31&lt;=0,L31&lt;=0),"n.m.",L31/K31-1)</f>
         <v>-0.234728729059324</v>
       </c>
       <c r="M32" s="16" t="n">
-        <f aca="false">IF(L31&lt;=0,"n.m.",M31/L31-1)</f>
+        <f aca="false">IF(OR(L31&lt;=0,M31&lt;=0),"n.m.",M31/L31-1)</f>
         <v>0.557409774301032</v>
       </c>
     </row>
@@ -16332,40 +16496,40 @@
       <c r="B40" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="E40" s="16" t="n">
-        <f aca="false">IF(D39&lt;=0,"n.m.",E39/D39-1)</f>
-        <v>-1.53293413173653</v>
+      <c r="E40" s="16" t="str">
+        <f aca="false">IF(OR(D39&lt;=0,E39&lt;=0),"n.m.",E39/D39-1)</f>
+        <v>n.m.</v>
       </c>
       <c r="F40" s="16" t="str">
-        <f aca="false">IF(E39&lt;=0,"n.m.",F39/E39-1)</f>
+        <f aca="false">IF(OR(E39&lt;=0,F39&lt;=0),"n.m.",F39/E39-1)</f>
         <v>n.m.</v>
       </c>
       <c r="G40" s="16" t="n">
-        <f aca="false">IF(F39&lt;=0,"n.m.",G39/F39-1)</f>
+        <f aca="false">IF(OR(F39&lt;=0,G39&lt;=0),"n.m.",G39/F39-1)</f>
         <v>5.37692307692308</v>
       </c>
       <c r="H40" s="16" t="n">
-        <f aca="false">IF(G39&lt;=0,"n.m.",H39/G39-1)</f>
+        <f aca="false">IF(OR(G39&lt;=0,H39&lt;=0),"n.m.",H39/G39-1)</f>
         <v>8.10977080820265</v>
       </c>
       <c r="I40" s="16" t="n">
-        <f aca="false">IF(H39&lt;=0,"n.m.",I39/H39-1)</f>
+        <f aca="false">IF(OR(H39&lt;=0,I39&lt;=0),"n.m.",I39/H39-1)</f>
         <v>1.32726534098006</v>
       </c>
       <c r="J40" s="16" t="n">
-        <f aca="false">IF(I39&lt;=0,"n.m.",J39/I39-1)</f>
+        <f aca="false">IF(OR(I39&lt;=0,J39&lt;=0),"n.m.",J39/I39-1)</f>
         <v>0.20646843818144</v>
       </c>
       <c r="K40" s="16" t="n">
-        <f aca="false">IF(J39&lt;=0,"n.m.",K39/J39-1)</f>
+        <f aca="false">IF(OR(J39&lt;=0,K39&lt;=0),"n.m.",K39/J39-1)</f>
         <v>-0.274776954863995</v>
       </c>
       <c r="L40" s="16" t="n">
-        <f aca="false">IF(K39&lt;=0,"n.m.",L39/K39-1)</f>
+        <f aca="false">IF(OR(K39&lt;=0,L39&lt;=0),"n.m.",L39/K39-1)</f>
         <v>-0.228837459801241</v>
       </c>
       <c r="M40" s="16" t="n">
-        <f aca="false">IF(L39&lt;=0,"n.m.",M39/L39-1)</f>
+        <f aca="false">IF(OR(L39&lt;=0,M39&lt;=0),"n.m.",M39/L39-1)</f>
         <v>0.550450938849317</v>
       </c>
     </row>
@@ -21450,29 +21614,29 @@
         <v>417</v>
       </c>
       <c r="D63" s="70" t="n">
-        <f aca="false">$I$57+(0-2)*$E$61</f>
+        <f aca="false">$I$57+(-2)*$E$61</f>
         <v>0.02</v>
       </c>
       <c r="E63" s="70" t="n">
-        <f aca="false">$I$57+(1-2)*$E$61</f>
+        <f aca="false">$I$57+(-1)*$E$61</f>
         <v>0.025</v>
       </c>
       <c r="F63" s="70" t="n">
-        <f aca="false">$I$57+(2-2)*$E$61</f>
+        <f aca="false">$I$57+(0)*$E$61</f>
         <v>0.03</v>
       </c>
       <c r="G63" s="70" t="n">
-        <f aca="false">$I$57+(3-2)*$E$61</f>
+        <f aca="false">$I$57+(1)*$E$61</f>
         <v>0.035</v>
       </c>
       <c r="H63" s="70" t="n">
-        <f aca="false">$I$57+(4-2)*$E$61</f>
+        <f aca="false">$I$57+(2)*$E$61</f>
         <v>0.04</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C64" s="71" t="n">
-        <f aca="false">$I$56+(0-2)*$C$61</f>
+        <f aca="false">$I$56+(-2)*$C$61</f>
         <v>0.118743575</v>
       </c>
       <c r="D64" s="72" t="n">
@@ -21498,7 +21662,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C65" s="71" t="n">
-        <f aca="false">$I$56+(1-2)*$C$61</f>
+        <f aca="false">$I$56+(-1)*$C$61</f>
         <v>0.123743575</v>
       </c>
       <c r="D65" s="72" t="n">
@@ -21524,7 +21688,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C66" s="71" t="n">
-        <f aca="false">$I$56+(2-2)*$C$61</f>
+        <f aca="false">$I$56+(0)*$C$61</f>
         <v>0.128743575</v>
       </c>
       <c r="D66" s="72" t="n">
@@ -21550,7 +21714,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C67" s="71" t="n">
-        <f aca="false">$I$56+(3-2)*$C$61</f>
+        <f aca="false">$I$56+(1)*$C$61</f>
         <v>0.133743575</v>
       </c>
       <c r="D67" s="72" t="n">
@@ -21576,7 +21740,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C68" s="71" t="n">
-        <f aca="false">$I$56+(4-2)*$C$61</f>
+        <f aca="false">$I$56+(2)*$C$61</f>
         <v>0.138743575</v>
       </c>
       <c r="D68" s="72" t="n">
@@ -21623,29 +21787,29 @@
         <v>420</v>
       </c>
       <c r="D73" s="70" t="n">
-        <f aca="false">$N$7+(0-2)*$G$61</f>
+        <f aca="false">$N$7+(-2)*$G$61</f>
         <v>0.58</v>
       </c>
       <c r="E73" s="70" t="n">
-        <f aca="false">$N$7+(1-2)*$G$61</f>
+        <f aca="false">$N$7+(-1)*$G$61</f>
         <v>0.6</v>
       </c>
       <c r="F73" s="70" t="n">
-        <f aca="false">$N$7+(2-2)*$G$61</f>
+        <f aca="false">$N$7+(0)*$G$61</f>
         <v>0.62</v>
       </c>
       <c r="G73" s="70" t="n">
-        <f aca="false">$N$7+(3-2)*$G$61</f>
+        <f aca="false">$N$7+(1)*$G$61</f>
         <v>0.64</v>
       </c>
       <c r="H73" s="70" t="n">
-        <f aca="false">$N$7+(4-2)*$G$61</f>
+        <f aca="false">$N$7+(2)*$G$61</f>
         <v>0.66</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C74" s="71" t="n">
-        <f aca="false">$I$56+(0-2)*$C$61</f>
+        <f aca="false">$I$56+(-2)*$C$61</f>
         <v>0.118743575</v>
       </c>
       <c r="D74" s="72" t="n">
@@ -21671,7 +21835,7 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C75" s="71" t="n">
-        <f aca="false">$I$56+(1-2)*$C$61</f>
+        <f aca="false">$I$56+(-1)*$C$61</f>
         <v>0.123743575</v>
       </c>
       <c r="D75" s="72" t="n">
@@ -21697,7 +21861,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C76" s="71" t="n">
-        <f aca="false">$I$56+(2-2)*$C$61</f>
+        <f aca="false">$I$56+(0)*$C$61</f>
         <v>0.128743575</v>
       </c>
       <c r="D76" s="72" t="n">
@@ -21723,7 +21887,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C77" s="71" t="n">
-        <f aca="false">$I$56+(3-2)*$C$61</f>
+        <f aca="false">$I$56+(1)*$C$61</f>
         <v>0.133743575</v>
       </c>
       <c r="D77" s="72" t="n">
@@ -21749,7 +21913,7 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C78" s="71" t="n">
-        <f aca="false">$I$56+(4-2)*$C$61</f>
+        <f aca="false">$I$56+(2)*$C$61</f>
         <v>0.138743575</v>
       </c>
       <c r="D78" s="72" t="n">
@@ -21935,15 +22099,15 @@
         <v>433</v>
       </c>
       <c r="D15" s="20" t="n">
-        <f aca="false">$D$10/DRE!H16</f>
+        <f aca="false">IF(DRE!H16&lt;=0,"n.m.",$D$10/DRE!H16)</f>
         <v>10.2217966097958</v>
       </c>
       <c r="E15" s="20" t="n">
-        <f aca="false">$D$10/DRE!I16</f>
+        <f aca="false">IF(DRE!I16&lt;=0,"n.m.",$D$10/DRE!I16)</f>
         <v>4.64676872371512</v>
       </c>
       <c r="F15" s="20" t="n">
-        <f aca="false">$D$10/DRE!J16</f>
+        <f aca="false">IF(DRE!J16&lt;=0,"n.m.",$D$10/DRE!J16)</f>
         <v>4.20087012475494</v>
       </c>
     </row>
@@ -21952,15 +22116,15 @@
         <v>434</v>
       </c>
       <c r="D16" s="20" t="n">
-        <f aca="false">$D$5/DRE!H31</f>
+        <f aca="false">IF(DRE!H31&lt;=0,"n.m.",$D$5/DRE!H31)</f>
         <v>14.0664603793892</v>
       </c>
       <c r="E16" s="20" t="n">
-        <f aca="false">$D$5/DRE!I31</f>
+        <f aca="false">IF(DRE!I31&lt;=0,"n.m.",$D$5/DRE!I31)</f>
         <v>6.00050177526336</v>
       </c>
       <c r="F16" s="20" t="n">
-        <f aca="false">$D$5/DRE!J31</f>
+        <f aca="false">IF(DRE!J31&lt;=0,"n.m.",$D$5/DRE!J31)</f>
         <v>4.97540359635524</v>
       </c>
     </row>
@@ -21969,15 +22133,15 @@
         <v>435</v>
       </c>
       <c r="D17" s="20" t="n">
-        <f aca="false">$D$5/DRE!H39</f>
+        <f aca="false">IF(DRE!H39&lt;=0,"n.m.",$D$5/DRE!H39)</f>
         <v>13.8448093220339</v>
       </c>
       <c r="E17" s="20" t="n">
-        <f aca="false">$D$5/DRE!I39</f>
+        <f aca="false">IF(DRE!I39&lt;=0,"n.m.",$D$5/DRE!I39)</f>
         <v>5.94896038635783</v>
       </c>
       <c r="F17" s="20" t="n">
-        <f aca="false">$D$5/DRE!J39</f>
+        <f aca="false">IF(DRE!J39&lt;=0,"n.m.",$D$5/DRE!J39)</f>
         <v>4.93088770339068</v>
       </c>
     </row>

</xml_diff>